<commit_message>
Getting acturate scores now.
</commit_message>
<xml_diff>
--- a/src/tools/rating_calculator/data/umamusume_rating_calculator.xlsx
+++ b/src/tools/rating_calculator/data/umamusume_rating_calculator.xlsx
@@ -3438,7 +3438,7 @@
     <xdr:ext cx="1981200" cy="1057275"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.png" title="Image"/>
+        <xdr:cNvPr id="0" name="image2.png" title="Image"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -3466,7 +3466,7 @@
     <xdr:ext cx="2876550" cy="2933700"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png" title="Image"/>
+        <xdr:cNvPr id="0" name="image1.png" title="Image"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -3515,7 +3515,7 @@
     <xdr:ext cx="3457575" cy="2828925"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image13.png" title="Image"/>
+        <xdr:cNvPr id="0" name="image12.png" title="Image"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -3543,7 +3543,7 @@
     <xdr:ext cx="1885950" cy="285750"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image11.png" title="Image"/>
+        <xdr:cNvPr id="0" name="image15.png" title="Image"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -3571,7 +3571,7 @@
     <xdr:ext cx="3619500" cy="1400175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image14.png" title="Image"/>
+        <xdr:cNvPr id="0" name="image13.png" title="Image"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -3599,7 +3599,7 @@
     <xdr:ext cx="5448300" cy="1400175"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image12.png" title="Image"/>
+        <xdr:cNvPr id="0" name="image11.png" title="Image"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -3627,7 +3627,7 @@
     <xdr:ext cx="6143625" cy="4057650"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image16.png" title="Image"/>
+        <xdr:cNvPr id="0" name="image14.png" title="Image"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -3711,7 +3711,7 @@
     <xdr:ext cx="952500" cy="952500"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image15.png"/>
+        <xdr:cNvPr id="0" name="image16.png"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -3744,7 +3744,7 @@
     <xdr:ext cx="962025" cy="76200"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image5.png"/>
+        <xdr:cNvPr id="0" name="image7.png"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -3800,7 +3800,7 @@
     <xdr:ext cx="962025" cy="76200"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image8.png"/>
+        <xdr:cNvPr id="0" name="image6.png"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -3828,7 +3828,7 @@
     <xdr:ext cx="962025" cy="190500"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image7.png"/>
+        <xdr:cNvPr id="0" name="image5.png"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -3856,7 +3856,7 @@
     <xdr:ext cx="962025" cy="190500"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image9.png"/>
+        <xdr:cNvPr id="0" name="image8.png"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -3884,7 +3884,7 @@
     <xdr:ext cx="962025" cy="190500"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image6.png"/>
+        <xdr:cNvPr id="0" name="image9.png"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -3917,7 +3917,7 @@
     <xdr:ext cx="10001250" cy="7429500"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image20.jpg" title="Image"/>
+        <xdr:cNvPr id="0" name="image19.jpg" title="Image"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -3978,7 +3978,7 @@
     <xdr:ext cx="10544175" cy="7829550"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image19.jpg" title="Image"/>
+        <xdr:cNvPr id="0" name="image20.jpg" title="Image"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>

</xml_diff>